<commit_message>
Denver: Garrett was 6 from 6, not 6 from 8 — data-entry error
Two "shot missed" events three seconds apart (H2 07:40 and 07:43, immediately
before his goal at 07:49) were a double-tap at the scorer's table. Removed, and
the play-by-play renumbered so the record reads as if the mis-entry never
happened.

Corrected in all three places that carry the number, so no two sheets can
disagree:
  Player Stats  Garrett 8 -> 6 shots, 75% -> 100%;  TEAM 57 -> 55, 68.4 -> 70.9
  Team Totals   Shots 57 -> 55, Shot % 68.4 -> 70.9
  Play-by-Play  154 -> 152 events

His goals, points and every other stat are unchanged, and he has no shot-map
markers, so nothing there to remove. The match report on the landing page now
reads "39 from 55 shots, a shooting rate of 71 per cent".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/games/AFA_Handball_vs_Denver_2026-08-22.xlsx
+++ b/games/AFA_Handball_vs_Denver_2026-08-22.xlsx
@@ -843,10 +843,10 @@
         <v>6</v>
       </c>
       <c r="E6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F6">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G6">
         <v>1</v>
@@ -1403,10 +1403,10 @@
         <v>39</v>
       </c>
       <c r="E16">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F16">
-        <v>68.4</v>
+        <v>70.9</v>
       </c>
       <c r="G16">
         <v>7</v>
@@ -1581,7 +1581,7 @@
         <v>Shots</v>
       </c>
       <c r="B3">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C3">
         <v>70</v>
@@ -1592,7 +1592,7 @@
         <v>Shot %</v>
       </c>
       <c r="B4">
-        <v>68.4</v>
+        <v>70.9</v>
       </c>
       <c r="C4">
         <v>57.1</v>
@@ -1695,7 +1695,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K155"/>
+  <dimension ref="A1:K153"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5275,7 +5275,7 @@
         <v>H2</v>
       </c>
       <c r="C103" t="str">
-        <v>07:40</v>
+        <v>07:49</v>
       </c>
       <c r="D103" t="str">
         <v>Air Force</v>
@@ -5287,13 +5287,13 @@
         <v>C1C Robert W. Garrett IV</v>
       </c>
       <c r="G103" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H103" t="str">
         <v/>
       </c>
       <c r="I103" t="str">
-        <v>24-21</v>
+        <v>25-21</v>
       </c>
       <c r="J103" t="str">
         <v/>
@@ -5310,25 +5310,25 @@
         <v>H2</v>
       </c>
       <c r="C104" t="str">
-        <v>07:43</v>
+        <v>08:54</v>
       </c>
       <c r="D104" t="str">
         <v>Air Force</v>
       </c>
       <c r="E104">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F104" t="str">
-        <v>C1C Robert W. Garrett IV</v>
+        <v>C1C Jack P. Tierney</v>
       </c>
       <c r="G104" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H104" t="str">
         <v/>
       </c>
       <c r="I104" t="str">
-        <v>24-21</v>
+        <v>26-21</v>
       </c>
       <c r="J104" t="str">
         <v/>
@@ -5345,16 +5345,16 @@
         <v>H2</v>
       </c>
       <c r="C105" t="str">
-        <v>07:49</v>
+        <v>09:13</v>
       </c>
       <c r="D105" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E105">
-        <v>5</v>
+        <v>Denver</v>
+      </c>
+      <c r="E105" t="str">
+        <v/>
       </c>
       <c r="F105" t="str">
-        <v>C1C Robert W. Garrett IV</v>
+        <v>Denver</v>
       </c>
       <c r="G105" t="str">
         <v>GOAL</v>
@@ -5363,13 +5363,13 @@
         <v/>
       </c>
       <c r="I105" t="str">
-        <v>25-21</v>
-      </c>
-      <c r="J105" t="str">
-        <v/>
-      </c>
-      <c r="K105" t="str">
-        <v/>
+        <v>26-22</v>
+      </c>
+      <c r="J105">
+        <v>79.1</v>
+      </c>
+      <c r="K105">
+        <v>68.2</v>
       </c>
     </row>
     <row r="106">
@@ -5380,16 +5380,16 @@
         <v>H2</v>
       </c>
       <c r="C106" t="str">
-        <v>08:54</v>
+        <v>09:24</v>
       </c>
       <c r="D106" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E106">
-        <v>1</v>
+        <v>Denver</v>
+      </c>
+      <c r="E106" t="str">
+        <v/>
       </c>
       <c r="F106" t="str">
-        <v>C1C Jack P. Tierney</v>
+        <v>Denver</v>
       </c>
       <c r="G106" t="str">
         <v>GOAL</v>
@@ -5398,13 +5398,13 @@
         <v/>
       </c>
       <c r="I106" t="str">
-        <v>26-21</v>
-      </c>
-      <c r="J106" t="str">
-        <v/>
-      </c>
-      <c r="K106" t="str">
-        <v/>
+        <v>26-23</v>
+      </c>
+      <c r="J106">
+        <v>16.5</v>
+      </c>
+      <c r="K106">
+        <v>44.9</v>
       </c>
     </row>
     <row r="107">
@@ -5415,7 +5415,7 @@
         <v>H2</v>
       </c>
       <c r="C107" t="str">
-        <v>09:13</v>
+        <v>09:27</v>
       </c>
       <c r="D107" t="str">
         <v>Denver</v>
@@ -5433,13 +5433,13 @@
         <v/>
       </c>
       <c r="I107" t="str">
-        <v>26-22</v>
+        <v>26-24</v>
       </c>
       <c r="J107">
-        <v>79.1</v>
+        <v>84.5</v>
       </c>
       <c r="K107">
-        <v>68.2</v>
+        <v>39</v>
       </c>
     </row>
     <row r="108">
@@ -5450,7 +5450,7 @@
         <v>H2</v>
       </c>
       <c r="C108" t="str">
-        <v>09:24</v>
+        <v>09:32</v>
       </c>
       <c r="D108" t="str">
         <v>Denver</v>
@@ -5468,13 +5468,13 @@
         <v/>
       </c>
       <c r="I108" t="str">
-        <v>26-23</v>
+        <v>26-25</v>
       </c>
       <c r="J108">
-        <v>16.5</v>
+        <v>84.2</v>
       </c>
       <c r="K108">
-        <v>44.9</v>
+        <v>77.8</v>
       </c>
     </row>
     <row r="109">
@@ -5485,7 +5485,7 @@
         <v>H2</v>
       </c>
       <c r="C109" t="str">
-        <v>09:27</v>
+        <v>10:24</v>
       </c>
       <c r="D109" t="str">
         <v>Denver</v>
@@ -5497,19 +5497,19 @@
         <v>Denver</v>
       </c>
       <c r="G109" t="str">
-        <v>GOAL</v>
+        <v>shot missed</v>
       </c>
       <c r="H109" t="str">
         <v/>
       </c>
       <c r="I109" t="str">
-        <v>26-24</v>
+        <v>26-25</v>
       </c>
       <c r="J109">
-        <v>84.5</v>
+        <v>51.5</v>
       </c>
       <c r="K109">
-        <v>39</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="110">
@@ -5520,19 +5520,19 @@
         <v>H2</v>
       </c>
       <c r="C110" t="str">
-        <v>09:32</v>
+        <v>10:29</v>
       </c>
       <c r="D110" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E110" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E110">
+        <v>10</v>
       </c>
       <c r="F110" t="str">
-        <v>Denver</v>
+        <v>C3C Evan M. Feller</v>
       </c>
       <c r="G110" t="str">
-        <v>GOAL</v>
+        <v>assist</v>
       </c>
       <c r="H110" t="str">
         <v/>
@@ -5540,11 +5540,11 @@
       <c r="I110" t="str">
         <v>26-25</v>
       </c>
-      <c r="J110">
-        <v>84.2</v>
-      </c>
-      <c r="K110">
-        <v>77.8</v>
+      <c r="J110" t="str">
+        <v/>
+      </c>
+      <c r="K110" t="str">
+        <v/>
       </c>
     </row>
     <row r="111">
@@ -5555,16 +5555,16 @@
         <v>H2</v>
       </c>
       <c r="C111" t="str">
-        <v>10:24</v>
+        <v>11:10</v>
       </c>
       <c r="D111" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E111" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E111">
+        <v>1</v>
       </c>
       <c r="F111" t="str">
-        <v>Denver</v>
+        <v>C1C Jack P. Tierney</v>
       </c>
       <c r="G111" t="str">
         <v>shot missed</v>
@@ -5575,11 +5575,11 @@
       <c r="I111" t="str">
         <v>26-25</v>
       </c>
-      <c r="J111">
-        <v>51.5</v>
-      </c>
-      <c r="K111">
-        <v>13.5</v>
+      <c r="J111" t="str">
+        <v/>
+      </c>
+      <c r="K111" t="str">
+        <v/>
       </c>
     </row>
     <row r="112">
@@ -5590,19 +5590,19 @@
         <v>H2</v>
       </c>
       <c r="C112" t="str">
-        <v>10:29</v>
+        <v>11:31</v>
       </c>
       <c r="D112" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E112">
-        <v>10</v>
+        <v>Denver</v>
+      </c>
+      <c r="E112" t="str">
+        <v/>
       </c>
       <c r="F112" t="str">
-        <v>C3C Evan M. Feller</v>
+        <v>Denver</v>
       </c>
       <c r="G112" t="str">
-        <v>assist</v>
+        <v>shot missed</v>
       </c>
       <c r="H112" t="str">
         <v/>
@@ -5610,11 +5610,11 @@
       <c r="I112" t="str">
         <v>26-25</v>
       </c>
-      <c r="J112" t="str">
-        <v/>
-      </c>
-      <c r="K112" t="str">
-        <v/>
+      <c r="J112">
+        <v>87.4</v>
+      </c>
+      <c r="K112">
+        <v>44.9</v>
       </c>
     </row>
     <row r="113">
@@ -5625,31 +5625,31 @@
         <v>H2</v>
       </c>
       <c r="C113" t="str">
-        <v>11:10</v>
+        <v>11:52</v>
       </c>
       <c r="D113" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E113">
-        <v>1</v>
+        <v>Denver</v>
+      </c>
+      <c r="E113" t="str">
+        <v/>
       </c>
       <c r="F113" t="str">
-        <v>C1C Jack P. Tierney</v>
+        <v>Denver</v>
       </c>
       <c r="G113" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H113" t="str">
         <v/>
       </c>
       <c r="I113" t="str">
-        <v>26-25</v>
-      </c>
-      <c r="J113" t="str">
-        <v/>
-      </c>
-      <c r="K113" t="str">
-        <v/>
+        <v>26-26</v>
+      </c>
+      <c r="J113">
+        <v>53.5</v>
+      </c>
+      <c r="K113">
+        <v>48.2</v>
       </c>
     </row>
     <row r="114">
@@ -5660,31 +5660,31 @@
         <v>H2</v>
       </c>
       <c r="C114" t="str">
-        <v>11:31</v>
+        <v>12:12</v>
       </c>
       <c r="D114" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E114" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E114">
+        <v>9</v>
       </c>
       <c r="F114" t="str">
-        <v>Denver</v>
+        <v>C3C Ian P. Cavendish</v>
       </c>
       <c r="G114" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H114" t="str">
         <v/>
       </c>
       <c r="I114" t="str">
-        <v>26-25</v>
-      </c>
-      <c r="J114">
-        <v>87.4</v>
-      </c>
-      <c r="K114">
-        <v>44.9</v>
+        <v>27-26</v>
+      </c>
+      <c r="J114" t="str">
+        <v/>
+      </c>
+      <c r="K114" t="str">
+        <v/>
       </c>
     </row>
     <row r="115">
@@ -5695,16 +5695,16 @@
         <v>H2</v>
       </c>
       <c r="C115" t="str">
-        <v>11:52</v>
+        <v>12:12</v>
       </c>
       <c r="D115" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E115" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E115">
+        <v>9</v>
       </c>
       <c r="F115" t="str">
-        <v>Denver</v>
+        <v>C3C Ian P. Cavendish</v>
       </c>
       <c r="G115" t="str">
         <v>GOAL</v>
@@ -5713,13 +5713,13 @@
         <v/>
       </c>
       <c r="I115" t="str">
-        <v>26-26</v>
-      </c>
-      <c r="J115">
-        <v>53.5</v>
-      </c>
-      <c r="K115">
-        <v>48.2</v>
+        <v>28-26</v>
+      </c>
+      <c r="J115" t="str">
+        <v/>
+      </c>
+      <c r="K115" t="str">
+        <v/>
       </c>
     </row>
     <row r="116">
@@ -5730,7 +5730,7 @@
         <v>H2</v>
       </c>
       <c r="C116" t="str">
-        <v>12:12</v>
+        <v>12:22</v>
       </c>
       <c r="D116" t="str">
         <v>Air Force</v>
@@ -5742,13 +5742,13 @@
         <v>C3C Ian P. Cavendish</v>
       </c>
       <c r="G116" t="str">
-        <v>GOAL</v>
+        <v>shot missed</v>
       </c>
       <c r="H116" t="str">
         <v/>
       </c>
       <c r="I116" t="str">
-        <v>27-26</v>
+        <v>28-26</v>
       </c>
       <c r="J116" t="str">
         <v/>
@@ -5765,7 +5765,7 @@
         <v>H2</v>
       </c>
       <c r="C117" t="str">
-        <v>12:12</v>
+        <v>12:24</v>
       </c>
       <c r="D117" t="str">
         <v>Air Force</v>
@@ -5777,7 +5777,7 @@
         <v>C3C Ian P. Cavendish</v>
       </c>
       <c r="G117" t="str">
-        <v>GOAL</v>
+        <v>shot missed</v>
       </c>
       <c r="H117" t="str">
         <v/>
@@ -5800,31 +5800,31 @@
         <v>H2</v>
       </c>
       <c r="C118" t="str">
-        <v>12:22</v>
+        <v>13:13</v>
       </c>
       <c r="D118" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E118">
-        <v>9</v>
+        <v>Denver</v>
+      </c>
+      <c r="E118" t="str">
+        <v/>
       </c>
       <c r="F118" t="str">
-        <v>C3C Ian P. Cavendish</v>
+        <v>Denver</v>
       </c>
       <c r="G118" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H118" t="str">
         <v/>
       </c>
       <c r="I118" t="str">
-        <v>28-26</v>
-      </c>
-      <c r="J118" t="str">
-        <v/>
-      </c>
-      <c r="K118" t="str">
-        <v/>
+        <v>28-27</v>
+      </c>
+      <c r="J118">
+        <v>66.4</v>
+      </c>
+      <c r="K118">
+        <v>81.1</v>
       </c>
     </row>
     <row r="119">
@@ -5835,25 +5835,25 @@
         <v>H2</v>
       </c>
       <c r="C119" t="str">
-        <v>12:24</v>
+        <v>13:23</v>
       </c>
       <c r="D119" t="str">
         <v>Air Force</v>
       </c>
       <c r="E119">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F119" t="str">
-        <v>C3C Ian P. Cavendish</v>
+        <v>C1C Ryan S. Sansano</v>
       </c>
       <c r="G119" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H119" t="str">
         <v/>
       </c>
       <c r="I119" t="str">
-        <v>28-26</v>
+        <v>29-27</v>
       </c>
       <c r="J119" t="str">
         <v/>
@@ -5870,7 +5870,7 @@
         <v>H2</v>
       </c>
       <c r="C120" t="str">
-        <v>13:13</v>
+        <v>13:34</v>
       </c>
       <c r="D120" t="str">
         <v>Denver</v>
@@ -5888,13 +5888,13 @@
         <v/>
       </c>
       <c r="I120" t="str">
-        <v>28-27</v>
+        <v>29-28</v>
       </c>
       <c r="J120">
-        <v>66.4</v>
+        <v>79.1</v>
       </c>
       <c r="K120">
-        <v>81.1</v>
+        <v>84.3</v>
       </c>
     </row>
     <row r="121">
@@ -5905,7 +5905,7 @@
         <v>H2</v>
       </c>
       <c r="C121" t="str">
-        <v>13:23</v>
+        <v>14:36</v>
       </c>
       <c r="D121" t="str">
         <v>Air Force</v>
@@ -5917,13 +5917,13 @@
         <v>C1C Ryan S. Sansano</v>
       </c>
       <c r="G121" t="str">
-        <v>GOAL</v>
+        <v>shot saved</v>
       </c>
       <c r="H121" t="str">
         <v/>
       </c>
       <c r="I121" t="str">
-        <v>29-27</v>
+        <v>29-28</v>
       </c>
       <c r="J121" t="str">
         <v/>
@@ -5940,7 +5940,7 @@
         <v>H2</v>
       </c>
       <c r="C122" t="str">
-        <v>13:34</v>
+        <v>15:01</v>
       </c>
       <c r="D122" t="str">
         <v>Denver</v>
@@ -5952,7 +5952,7 @@
         <v>Denver</v>
       </c>
       <c r="G122" t="str">
-        <v>GOAL</v>
+        <v>shot missed</v>
       </c>
       <c r="H122" t="str">
         <v/>
@@ -5961,10 +5961,10 @@
         <v>29-28</v>
       </c>
       <c r="J122">
-        <v>79.1</v>
+        <v>83.3</v>
       </c>
       <c r="K122">
-        <v>84.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="123">
@@ -5975,19 +5975,19 @@
         <v>H2</v>
       </c>
       <c r="C123" t="str">
-        <v>14:36</v>
+        <v>15:38</v>
       </c>
       <c r="D123" t="str">
         <v>Air Force</v>
       </c>
       <c r="E123">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F123" t="str">
-        <v>C1C Ryan S. Sansano</v>
+        <v>C3C Barrett S. Waldvogel</v>
       </c>
       <c r="G123" t="str">
-        <v>shot saved</v>
+        <v>shot missed</v>
       </c>
       <c r="H123" t="str">
         <v/>
@@ -6010,19 +6010,19 @@
         <v>H2</v>
       </c>
       <c r="C124" t="str">
-        <v>15:01</v>
+        <v>16:16</v>
       </c>
       <c r="D124" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E124" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E124">
+        <v>13</v>
       </c>
       <c r="F124" t="str">
-        <v>Denver</v>
+        <v>C3C Barrett S. Waldvogel</v>
       </c>
       <c r="G124" t="str">
-        <v>shot missed</v>
+        <v>turnover</v>
       </c>
       <c r="H124" t="str">
         <v/>
@@ -6030,11 +6030,11 @@
       <c r="I124" t="str">
         <v>29-28</v>
       </c>
-      <c r="J124">
-        <v>83.3</v>
-      </c>
-      <c r="K124">
-        <v>5.2</v>
+      <c r="J124" t="str">
+        <v/>
+      </c>
+      <c r="K124" t="str">
+        <v/>
       </c>
     </row>
     <row r="125">
@@ -6045,31 +6045,31 @@
         <v>H2</v>
       </c>
       <c r="C125" t="str">
-        <v>15:38</v>
+        <v>16:33</v>
       </c>
       <c r="D125" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E125">
-        <v>13</v>
+        <v>Denver</v>
+      </c>
+      <c r="E125" t="str">
+        <v/>
       </c>
       <c r="F125" t="str">
-        <v>C3C Barrett S. Waldvogel</v>
+        <v>Denver</v>
       </c>
       <c r="G125" t="str">
-        <v>shot missed</v>
+        <v>7m GOAL</v>
       </c>
       <c r="H125" t="str">
         <v/>
       </c>
       <c r="I125" t="str">
-        <v>29-28</v>
-      </c>
-      <c r="J125" t="str">
-        <v/>
-      </c>
-      <c r="K125" t="str">
-        <v/>
+        <v>29-29</v>
+      </c>
+      <c r="J125">
+        <v>77.9</v>
+      </c>
+      <c r="K125">
+        <v>39.9</v>
       </c>
     </row>
     <row r="126">
@@ -6080,25 +6080,25 @@
         <v>H2</v>
       </c>
       <c r="C126" t="str">
-        <v>16:16</v>
+        <v>16:33</v>
       </c>
       <c r="D126" t="str">
         <v>Air Force</v>
       </c>
       <c r="E126">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F126" t="str">
-        <v>C3C Barrett S. Waldvogel</v>
+        <v>C2C Roman E. Trice</v>
       </c>
       <c r="G126" t="str">
-        <v>turnover</v>
+        <v>GOAL</v>
       </c>
       <c r="H126" t="str">
         <v/>
       </c>
       <c r="I126" t="str">
-        <v>29-28</v>
+        <v>30-29</v>
       </c>
       <c r="J126" t="str">
         <v/>
@@ -6127,19 +6127,19 @@
         <v>Denver</v>
       </c>
       <c r="G127" t="str">
-        <v>7m GOAL</v>
+        <v>GOAL</v>
       </c>
       <c r="H127" t="str">
         <v/>
       </c>
       <c r="I127" t="str">
-        <v>29-29</v>
+        <v>30-30</v>
       </c>
       <c r="J127">
-        <v>77.9</v>
+        <v>16.7</v>
       </c>
       <c r="K127">
-        <v>39.9</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="128">
@@ -6156,19 +6156,19 @@
         <v>Air Force</v>
       </c>
       <c r="E128">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F128" t="str">
-        <v>C2C Roman E. Trice</v>
+        <v>C1C Logan T Cook</v>
       </c>
       <c r="G128" t="str">
-        <v>GOAL</v>
+        <v>2-minute</v>
       </c>
       <c r="H128" t="str">
         <v/>
       </c>
       <c r="I128" t="str">
-        <v>30-29</v>
+        <v>30-30</v>
       </c>
       <c r="J128" t="str">
         <v/>
@@ -6203,13 +6203,13 @@
         <v/>
       </c>
       <c r="I129" t="str">
-        <v>30-30</v>
+        <v>30-31</v>
       </c>
       <c r="J129">
-        <v>16.7</v>
+        <v>78.8</v>
       </c>
       <c r="K129">
-        <v>20.5</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="130">
@@ -6232,13 +6232,13 @@
         <v>C1C Logan T Cook</v>
       </c>
       <c r="G130" t="str">
-        <v>2-minute</v>
+        <v>GOAL</v>
       </c>
       <c r="H130" t="str">
         <v/>
       </c>
       <c r="I130" t="str">
-        <v>30-30</v>
+        <v>31-31</v>
       </c>
       <c r="J130" t="str">
         <v/>
@@ -6273,13 +6273,13 @@
         <v/>
       </c>
       <c r="I131" t="str">
-        <v>30-31</v>
+        <v>31-32</v>
       </c>
       <c r="J131">
-        <v>78.8</v>
+        <v>15.9</v>
       </c>
       <c r="K131">
-        <v>58.8</v>
+        <v>32</v>
       </c>
     </row>
     <row r="132">
@@ -6290,31 +6290,31 @@
         <v>H2</v>
       </c>
       <c r="C132" t="str">
-        <v>16:33</v>
+        <v>17:18</v>
       </c>
       <c r="D132" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E132">
-        <v>2</v>
+        <v>Denver</v>
+      </c>
+      <c r="E132" t="str">
+        <v/>
       </c>
       <c r="F132" t="str">
-        <v>C1C Logan T Cook</v>
+        <v>Denver</v>
       </c>
       <c r="G132" t="str">
-        <v>GOAL</v>
+        <v>shot saved — Air Force save</v>
       </c>
       <c r="H132" t="str">
         <v/>
       </c>
       <c r="I132" t="str">
-        <v>31-31</v>
-      </c>
-      <c r="J132" t="str">
-        <v/>
-      </c>
-      <c r="K132" t="str">
-        <v/>
+        <v>31-32</v>
+      </c>
+      <c r="J132">
+        <v>75.2</v>
+      </c>
+      <c r="K132">
+        <v>76.5</v>
       </c>
     </row>
     <row r="133">
@@ -6325,7 +6325,7 @@
         <v>H2</v>
       </c>
       <c r="C133" t="str">
-        <v>16:33</v>
+        <v>17:39</v>
       </c>
       <c r="D133" t="str">
         <v>Denver</v>
@@ -6343,13 +6343,13 @@
         <v/>
       </c>
       <c r="I133" t="str">
-        <v>31-32</v>
+        <v>31-33</v>
       </c>
       <c r="J133">
-        <v>15.9</v>
+        <v>68.5</v>
       </c>
       <c r="K133">
-        <v>32</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="134">
@@ -6360,7 +6360,7 @@
         <v>H2</v>
       </c>
       <c r="C134" t="str">
-        <v>17:18</v>
+        <v>18:50</v>
       </c>
       <c r="D134" t="str">
         <v>Denver</v>
@@ -6372,19 +6372,19 @@
         <v>Denver</v>
       </c>
       <c r="G134" t="str">
-        <v>shot saved — Air Force save</v>
+        <v>GOAL</v>
       </c>
       <c r="H134" t="str">
         <v/>
       </c>
       <c r="I134" t="str">
-        <v>31-32</v>
+        <v>31-34</v>
       </c>
       <c r="J134">
-        <v>75.2</v>
+        <v>23.3</v>
       </c>
       <c r="K134">
-        <v>76.5</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="135">
@@ -6395,16 +6395,16 @@
         <v>H2</v>
       </c>
       <c r="C135" t="str">
-        <v>17:39</v>
+        <v>19:24</v>
       </c>
       <c r="D135" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E135" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E135">
+        <v>8</v>
       </c>
       <c r="F135" t="str">
-        <v>Denver</v>
+        <v>C2C Roman E. Trice</v>
       </c>
       <c r="G135" t="str">
         <v>GOAL</v>
@@ -6413,13 +6413,13 @@
         <v/>
       </c>
       <c r="I135" t="str">
-        <v>31-33</v>
-      </c>
-      <c r="J135">
-        <v>68.5</v>
-      </c>
-      <c r="K135">
-        <v>17.4</v>
+        <v>32-34</v>
+      </c>
+      <c r="J135" t="str">
+        <v/>
+      </c>
+      <c r="K135" t="str">
+        <v/>
       </c>
     </row>
     <row r="136">
@@ -6430,7 +6430,7 @@
         <v>H2</v>
       </c>
       <c r="C136" t="str">
-        <v>18:50</v>
+        <v>20:02</v>
       </c>
       <c r="D136" t="str">
         <v>Denver</v>
@@ -6448,13 +6448,13 @@
         <v/>
       </c>
       <c r="I136" t="str">
-        <v>31-34</v>
+        <v>32-35</v>
       </c>
       <c r="J136">
-        <v>23.3</v>
+        <v>17</v>
       </c>
       <c r="K136">
-        <v>51.9</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="137">
@@ -6465,16 +6465,16 @@
         <v>H2</v>
       </c>
       <c r="C137" t="str">
-        <v>19:24</v>
+        <v>20:33</v>
       </c>
       <c r="D137" t="str">
         <v>Air Force</v>
       </c>
       <c r="E137">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F137" t="str">
-        <v>C2C Roman E. Trice</v>
+        <v>C3C Sean W. Windell</v>
       </c>
       <c r="G137" t="str">
         <v>GOAL</v>
@@ -6483,7 +6483,7 @@
         <v/>
       </c>
       <c r="I137" t="str">
-        <v>32-34</v>
+        <v>33-35</v>
       </c>
       <c r="J137" t="str">
         <v/>
@@ -6500,7 +6500,7 @@
         <v>H2</v>
       </c>
       <c r="C138" t="str">
-        <v>20:02</v>
+        <v>21:02</v>
       </c>
       <c r="D138" t="str">
         <v>Denver</v>
@@ -6512,19 +6512,19 @@
         <v>Denver</v>
       </c>
       <c r="G138" t="str">
-        <v>GOAL</v>
+        <v>shot missed</v>
       </c>
       <c r="H138" t="str">
         <v/>
       </c>
       <c r="I138" t="str">
-        <v>32-35</v>
+        <v>33-35</v>
       </c>
       <c r="J138">
-        <v>17</v>
+        <v>56.8</v>
       </c>
       <c r="K138">
-        <v>66.5</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="139">
@@ -6535,19 +6535,19 @@
         <v>H2</v>
       </c>
       <c r="C139" t="str">
-        <v>20:33</v>
+        <v>21:23</v>
       </c>
       <c r="D139" t="str">
         <v>Air Force</v>
       </c>
       <c r="E139">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="F139" t="str">
-        <v>C3C Sean W. Windell</v>
+        <v>C1C Jack P. Tierney</v>
       </c>
       <c r="G139" t="str">
-        <v>GOAL</v>
+        <v>shot missed</v>
       </c>
       <c r="H139" t="str">
         <v/>
@@ -6570,7 +6570,7 @@
         <v>H2</v>
       </c>
       <c r="C140" t="str">
-        <v>21:02</v>
+        <v>21:46</v>
       </c>
       <c r="D140" t="str">
         <v>Denver</v>
@@ -6582,19 +6582,19 @@
         <v>Denver</v>
       </c>
       <c r="G140" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H140" t="str">
         <v/>
       </c>
       <c r="I140" t="str">
-        <v>33-35</v>
+        <v>33-36</v>
       </c>
       <c r="J140">
-        <v>56.8</v>
+        <v>81.1</v>
       </c>
       <c r="K140">
-        <v>14.2</v>
+        <v>71.3</v>
       </c>
     </row>
     <row r="141">
@@ -6605,25 +6605,25 @@
         <v>H2</v>
       </c>
       <c r="C141" t="str">
-        <v>21:23</v>
+        <v>22:30</v>
       </c>
       <c r="D141" t="str">
         <v>Air Force</v>
       </c>
       <c r="E141">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F141" t="str">
-        <v>C1C Jack P. Tierney</v>
+        <v>C1C Troy E. Miller</v>
       </c>
       <c r="G141" t="str">
-        <v>shot missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H141" t="str">
         <v/>
       </c>
       <c r="I141" t="str">
-        <v>33-35</v>
+        <v>34-36</v>
       </c>
       <c r="J141" t="str">
         <v/>
@@ -6640,7 +6640,7 @@
         <v>H2</v>
       </c>
       <c r="C142" t="str">
-        <v>21:46</v>
+        <v>23:32</v>
       </c>
       <c r="D142" t="str">
         <v>Denver</v>
@@ -6652,19 +6652,19 @@
         <v>Denver</v>
       </c>
       <c r="G142" t="str">
-        <v>GOAL</v>
+        <v>shot missed</v>
       </c>
       <c r="H142" t="str">
         <v/>
       </c>
       <c r="I142" t="str">
-        <v>33-36</v>
+        <v>34-36</v>
       </c>
       <c r="J142">
-        <v>81.1</v>
+        <v>5</v>
       </c>
       <c r="K142">
-        <v>71.3</v>
+        <v>52.3</v>
       </c>
     </row>
     <row r="143">
@@ -6675,16 +6675,16 @@
         <v>H2</v>
       </c>
       <c r="C143" t="str">
-        <v>22:30</v>
+        <v>23:41</v>
       </c>
       <c r="D143" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E143">
-        <v>6</v>
+        <v>Denver</v>
+      </c>
+      <c r="E143" t="str">
+        <v/>
       </c>
       <c r="F143" t="str">
-        <v>C1C Troy E. Miller</v>
+        <v>Denver</v>
       </c>
       <c r="G143" t="str">
         <v>GOAL</v>
@@ -6693,13 +6693,13 @@
         <v/>
       </c>
       <c r="I143" t="str">
-        <v>34-36</v>
-      </c>
-      <c r="J143" t="str">
-        <v/>
-      </c>
-      <c r="K143" t="str">
-        <v/>
+        <v>34-37</v>
+      </c>
+      <c r="J143">
+        <v>77.3</v>
+      </c>
+      <c r="K143">
+        <v>22</v>
       </c>
     </row>
     <row r="144">
@@ -6710,31 +6710,31 @@
         <v>H2</v>
       </c>
       <c r="C144" t="str">
-        <v>23:32</v>
+        <v>23:49</v>
       </c>
       <c r="D144" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E144" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E144">
+        <v>5</v>
       </c>
       <c r="F144" t="str">
-        <v>Denver</v>
+        <v>C1C Robert W. Garrett IV</v>
       </c>
       <c r="G144" t="str">
-        <v>shot missed</v>
+        <v>turnover</v>
       </c>
       <c r="H144" t="str">
         <v/>
       </c>
       <c r="I144" t="str">
-        <v>34-36</v>
-      </c>
-      <c r="J144">
-        <v>5</v>
-      </c>
-      <c r="K144">
-        <v>52.3</v>
+        <v>34-37</v>
+      </c>
+      <c r="J144" t="str">
+        <v/>
+      </c>
+      <c r="K144" t="str">
+        <v/>
       </c>
     </row>
     <row r="145">
@@ -6745,16 +6745,16 @@
         <v>H2</v>
       </c>
       <c r="C145" t="str">
-        <v>23:41</v>
+        <v>23:51</v>
       </c>
       <c r="D145" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E145" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E145">
+        <v>1</v>
       </c>
       <c r="F145" t="str">
-        <v>Denver</v>
+        <v>C1C Jack P. Tierney</v>
       </c>
       <c r="G145" t="str">
         <v>GOAL</v>
@@ -6763,13 +6763,13 @@
         <v/>
       </c>
       <c r="I145" t="str">
-        <v>34-37</v>
-      </c>
-      <c r="J145">
-        <v>77.3</v>
-      </c>
-      <c r="K145">
-        <v>22</v>
+        <v>35-37</v>
+      </c>
+      <c r="J145" t="str">
+        <v/>
+      </c>
+      <c r="K145" t="str">
+        <v/>
       </c>
     </row>
     <row r="146">
@@ -6780,25 +6780,25 @@
         <v>H2</v>
       </c>
       <c r="C146" t="str">
-        <v>23:49</v>
+        <v>24:40</v>
       </c>
       <c r="D146" t="str">
         <v>Air Force</v>
       </c>
       <c r="E146">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F146" t="str">
-        <v>C1C Robert W. Garrett IV</v>
+        <v>C3C Evan M. Feller</v>
       </c>
       <c r="G146" t="str">
-        <v>turnover</v>
+        <v>GOAL</v>
       </c>
       <c r="H146" t="str">
         <v/>
       </c>
       <c r="I146" t="str">
-        <v>34-37</v>
+        <v>36-37</v>
       </c>
       <c r="J146" t="str">
         <v/>
@@ -6815,16 +6815,16 @@
         <v>H2</v>
       </c>
       <c r="C147" t="str">
-        <v>23:51</v>
+        <v>25:35</v>
       </c>
       <c r="D147" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E147">
-        <v>1</v>
+        <v>Denver</v>
+      </c>
+      <c r="E147" t="str">
+        <v/>
       </c>
       <c r="F147" t="str">
-        <v>C1C Jack P. Tierney</v>
+        <v>Denver</v>
       </c>
       <c r="G147" t="str">
         <v>GOAL</v>
@@ -6833,13 +6833,13 @@
         <v/>
       </c>
       <c r="I147" t="str">
-        <v>35-37</v>
-      </c>
-      <c r="J147" t="str">
-        <v/>
-      </c>
-      <c r="K147" t="str">
-        <v/>
+        <v>36-38</v>
+      </c>
+      <c r="J147">
+        <v>78.8</v>
+      </c>
+      <c r="K147">
+        <v>28.3</v>
       </c>
     </row>
     <row r="148">
@@ -6850,7 +6850,7 @@
         <v>H2</v>
       </c>
       <c r="C148" t="str">
-        <v>24:40</v>
+        <v>25:43</v>
       </c>
       <c r="D148" t="str">
         <v>Air Force</v>
@@ -6868,7 +6868,7 @@
         <v/>
       </c>
       <c r="I148" t="str">
-        <v>36-37</v>
+        <v>37-38</v>
       </c>
       <c r="J148" t="str">
         <v/>
@@ -6885,16 +6885,16 @@
         <v>H2</v>
       </c>
       <c r="C149" t="str">
-        <v>25:35</v>
+        <v>25:58</v>
       </c>
       <c r="D149" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E149" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E149">
+        <v>1</v>
       </c>
       <c r="F149" t="str">
-        <v>Denver</v>
+        <v>C1C Jack P. Tierney</v>
       </c>
       <c r="G149" t="str">
         <v>GOAL</v>
@@ -6903,13 +6903,13 @@
         <v/>
       </c>
       <c r="I149" t="str">
-        <v>36-38</v>
-      </c>
-      <c r="J149">
-        <v>78.8</v>
-      </c>
-      <c r="K149">
-        <v>28.3</v>
+        <v>38-38</v>
+      </c>
+      <c r="J149" t="str">
+        <v/>
+      </c>
+      <c r="K149" t="str">
+        <v/>
       </c>
     </row>
     <row r="150">
@@ -6920,16 +6920,16 @@
         <v>H2</v>
       </c>
       <c r="C150" t="str">
-        <v>25:43</v>
+        <v>26:26</v>
       </c>
       <c r="D150" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E150">
-        <v>10</v>
+        <v>Denver</v>
+      </c>
+      <c r="E150" t="str">
+        <v/>
       </c>
       <c r="F150" t="str">
-        <v>C3C Evan M. Feller</v>
+        <v>Denver</v>
       </c>
       <c r="G150" t="str">
         <v>GOAL</v>
@@ -6938,13 +6938,13 @@
         <v/>
       </c>
       <c r="I150" t="str">
-        <v>37-38</v>
-      </c>
-      <c r="J150" t="str">
-        <v/>
-      </c>
-      <c r="K150" t="str">
-        <v/>
+        <v>38-39</v>
+      </c>
+      <c r="J150">
+        <v>58.3</v>
+      </c>
+      <c r="K150">
+        <v>27</v>
       </c>
     </row>
     <row r="151">
@@ -6955,25 +6955,25 @@
         <v>H2</v>
       </c>
       <c r="C151" t="str">
-        <v>25:58</v>
+        <v>28:07</v>
       </c>
       <c r="D151" t="str">
         <v>Air Force</v>
       </c>
       <c r="E151">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F151" t="str">
-        <v>C1C Jack P. Tierney</v>
+        <v>C1C Ryan S. Sansano</v>
       </c>
       <c r="G151" t="str">
-        <v>GOAL</v>
+        <v>7m missed</v>
       </c>
       <c r="H151" t="str">
         <v/>
       </c>
       <c r="I151" t="str">
-        <v>38-38</v>
+        <v>38-39</v>
       </c>
       <c r="J151" t="str">
         <v/>
@@ -6990,16 +6990,16 @@
         <v>H2</v>
       </c>
       <c r="C152" t="str">
-        <v>26:26</v>
+        <v>28:17</v>
       </c>
       <c r="D152" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E152" t="str">
-        <v/>
+        <v>Air Force</v>
+      </c>
+      <c r="E152">
+        <v>5</v>
       </c>
       <c r="F152" t="str">
-        <v>Denver</v>
+        <v>C1C Robert W. Garrett IV</v>
       </c>
       <c r="G152" t="str">
         <v>GOAL</v>
@@ -7008,13 +7008,13 @@
         <v/>
       </c>
       <c r="I152" t="str">
-        <v>38-39</v>
-      </c>
-      <c r="J152">
-        <v>58.3</v>
-      </c>
-      <c r="K152">
-        <v>27</v>
+        <v>39-39</v>
+      </c>
+      <c r="J152" t="str">
+        <v/>
+      </c>
+      <c r="K152" t="str">
+        <v/>
       </c>
     </row>
     <row r="153">
@@ -7025,106 +7025,36 @@
         <v>H2</v>
       </c>
       <c r="C153" t="str">
-        <v>28:07</v>
+        <v>28:47</v>
       </c>
       <c r="D153" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E153">
-        <v>3</v>
+        <v>Denver</v>
+      </c>
+      <c r="E153" t="str">
+        <v/>
       </c>
       <c r="F153" t="str">
-        <v>C1C Ryan S. Sansano</v>
+        <v>Denver</v>
       </c>
       <c r="G153" t="str">
-        <v>7m missed</v>
+        <v>GOAL</v>
       </c>
       <c r="H153" t="str">
         <v/>
       </c>
       <c r="I153" t="str">
-        <v>38-39</v>
-      </c>
-      <c r="J153" t="str">
-        <v/>
-      </c>
-      <c r="K153" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154">
-        <v>153</v>
-      </c>
-      <c r="B154" t="str">
-        <v>H2</v>
-      </c>
-      <c r="C154" t="str">
-        <v>28:17</v>
-      </c>
-      <c r="D154" t="str">
-        <v>Air Force</v>
-      </c>
-      <c r="E154">
-        <v>5</v>
-      </c>
-      <c r="F154" t="str">
-        <v>C1C Robert W. Garrett IV</v>
-      </c>
-      <c r="G154" t="str">
-        <v>GOAL</v>
-      </c>
-      <c r="H154" t="str">
-        <v/>
-      </c>
-      <c r="I154" t="str">
-        <v>39-39</v>
-      </c>
-      <c r="J154" t="str">
-        <v/>
-      </c>
-      <c r="K154" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155">
-        <v>154</v>
-      </c>
-      <c r="B155" t="str">
-        <v>H2</v>
-      </c>
-      <c r="C155" t="str">
-        <v>28:47</v>
-      </c>
-      <c r="D155" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="E155" t="str">
-        <v/>
-      </c>
-      <c r="F155" t="str">
-        <v>Denver</v>
-      </c>
-      <c r="G155" t="str">
-        <v>GOAL</v>
-      </c>
-      <c r="H155" t="str">
-        <v/>
-      </c>
-      <c r="I155" t="str">
         <v>39-40</v>
       </c>
-      <c r="J155">
+      <c r="J153">
         <v>73.2</v>
       </c>
-      <c r="K155">
+      <c r="K153">
         <v>79.3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K155"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K153"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Denver: three more assists for Garrett
Read as additive — 1 on the sheet plus 3, so he finishes with 4. Points move
with them (goals + assists in the exporter's own formula): Garrett 7 -> 10,
TEAM 46 -> 49, team assists 7 -> 10. Team Totals carries no assists row, so
nothing there can fall out of step.

The play-by-play still shows his one recorded assist event. The other three are
not in it deliberately: nobody recorded when they happened, and inventing three
timestamps would put moments into the game's timeline that were never observed.
Every display — the season tables, his card, the match report — reads assists
from Player Stats, so all of them show 4.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/games/AFA_Handball_vs_Denver_2026-08-22.xlsx
+++ b/games/AFA_Handball_vs_Denver_2026-08-22.xlsx
@@ -849,7 +849,7 @@
         <v>100</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -882,7 +882,7 @@
         <v>0</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -1409,7 +1409,7 @@
         <v>70.9</v>
       </c>
       <c r="G16">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H16">
         <v>2</v>
@@ -1442,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="R16">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>